<commit_message>
Inclusão do projeto de bot para Indicares
</commit_message>
<xml_diff>
--- a/dados_teste/Agrotóxicos.xlsx
+++ b/dados_teste/Agrotóxicos.xlsx
@@ -464,7 +464,7 @@
     <outlinePr summaryBelow="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G467"/>
+  <dimension ref="A1:G525"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13.57642857142857" bestFit="1" customWidth="1" style="9" min="1" max="1"/>
@@ -14935,6 +14935,1804 @@
         <v>2.478</v>
       </c>
     </row>
+    <row r="468">
+      <c r="A468" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B468" t="inlineStr">
+        <is>
+          <t>Inseticida</t>
+        </is>
+      </c>
+      <c r="C468" t="inlineStr">
+        <is>
+          <t>CLORPIRIFÓS</t>
+        </is>
+      </c>
+      <c r="D468" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="E468" t="n">
+        <v>52.23999999999999</v>
+      </c>
+      <c r="F468" t="inlineStr">
+        <is>
+          <t>Alface</t>
+        </is>
+      </c>
+      <c r="G468" t="n">
+        <v>2.272861111111111</v>
+      </c>
+    </row>
+    <row r="469">
+      <c r="A469" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B469" t="inlineStr">
+        <is>
+          <t>Inseticida</t>
+        </is>
+      </c>
+      <c r="C469" t="inlineStr">
+        <is>
+          <t>ENGEO PLENO, 106 G/L, TIAMETOXAM, NEONICOTINÓIDE + PIRETRÓIDE, SC</t>
+        </is>
+      </c>
+      <c r="D469" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="E469" t="n">
+        <v>183.335</v>
+      </c>
+      <c r="F469" t="inlineStr">
+        <is>
+          <t>Banana</t>
+        </is>
+      </c>
+      <c r="G469" t="n">
+        <v>2.6975</v>
+      </c>
+    </row>
+    <row r="470">
+      <c r="A470" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B470" t="inlineStr">
+        <is>
+          <t>Inseticida</t>
+        </is>
+      </c>
+      <c r="C470" t="inlineStr">
+        <is>
+          <t>IMIDACLOPRID 700, 700 G/KG, IMIDACLOPRIDO, NEONICOTINÓIDE, WG</t>
+        </is>
+      </c>
+      <c r="D470" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="E470" t="n">
+        <v>113.81</v>
+      </c>
+      <c r="F470" t="inlineStr">
+        <is>
+          <t>Alface</t>
+        </is>
+      </c>
+      <c r="G470" t="n">
+        <v>2.272861111111111</v>
+      </c>
+    </row>
+    <row r="471">
+      <c r="A471" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B471" t="inlineStr">
+        <is>
+          <t>Herbicida</t>
+        </is>
+      </c>
+      <c r="C471" t="inlineStr">
+        <is>
+          <t>DIURON, 500 SC</t>
+        </is>
+      </c>
+      <c r="D471" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="E471" t="n">
+        <v>55.1</v>
+      </c>
+      <c r="F471" t="inlineStr">
+        <is>
+          <t>Banana</t>
+        </is>
+      </c>
+      <c r="G471" t="n">
+        <v>2.698</v>
+      </c>
+    </row>
+    <row r="472">
+      <c r="A472" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B472" t="inlineStr">
+        <is>
+          <t>Herbicida</t>
+        </is>
+      </c>
+      <c r="C472" t="inlineStr">
+        <is>
+          <t>GLIFOSATO</t>
+        </is>
+      </c>
+      <c r="D472" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="E472" t="n">
+        <v>33.67</v>
+      </c>
+      <c r="F472" t="inlineStr">
+        <is>
+          <t>Alface</t>
+        </is>
+      </c>
+      <c r="G472" t="n">
+        <v>2.273</v>
+      </c>
+    </row>
+    <row r="473">
+      <c r="A473" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B473" t="inlineStr">
+        <is>
+          <t>Herbicida</t>
+        </is>
+      </c>
+      <c r="C473" t="inlineStr">
+        <is>
+          <t>2,4-D</t>
+        </is>
+      </c>
+      <c r="D473" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="E473" t="n">
+        <v>20.02</v>
+      </c>
+      <c r="F473" t="inlineStr">
+        <is>
+          <t>Banana</t>
+        </is>
+      </c>
+      <c r="G473" t="n">
+        <v>2.698</v>
+      </c>
+    </row>
+    <row r="474">
+      <c r="A474" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B474" t="inlineStr">
+        <is>
+          <t>Inseticida</t>
+        </is>
+      </c>
+      <c r="C474" t="inlineStr">
+        <is>
+          <t>CLORPIRIFÓS</t>
+        </is>
+      </c>
+      <c r="D474" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="E474" t="n">
+        <v>52.23999999999999</v>
+      </c>
+      <c r="F474" t="inlineStr">
+        <is>
+          <t>Alface</t>
+        </is>
+      </c>
+      <c r="G474" t="n">
+        <v>2.2805</v>
+      </c>
+    </row>
+    <row r="475">
+      <c r="A475" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B475" t="inlineStr">
+        <is>
+          <t>Inseticida</t>
+        </is>
+      </c>
+      <c r="C475" t="inlineStr">
+        <is>
+          <t>IMIDACLOPRID 700, 700 G/KG, IMIDACLOPRIDO, NEONICOTINÓIDE, WG</t>
+        </is>
+      </c>
+      <c r="D475" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="E475" t="n">
+        <v>113.81</v>
+      </c>
+      <c r="F475" t="inlineStr">
+        <is>
+          <t>Alface</t>
+        </is>
+      </c>
+      <c r="G475" t="n">
+        <v>2.2805</v>
+      </c>
+    </row>
+    <row r="476">
+      <c r="A476" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B476" t="inlineStr">
+        <is>
+          <t>Inseticida</t>
+        </is>
+      </c>
+      <c r="C476" t="inlineStr">
+        <is>
+          <t>ENGEO PLENO, 106 G/L, TIAMETOXAM, NEONICOTINÓIDE + PIRETRÓIDE, SC</t>
+        </is>
+      </c>
+      <c r="D476" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="E476" t="n">
+        <v>183.335</v>
+      </c>
+      <c r="F476" t="inlineStr">
+        <is>
+          <t>Banana</t>
+        </is>
+      </c>
+      <c r="G476" t="n">
+        <v>2.815833333333333</v>
+      </c>
+    </row>
+    <row r="477">
+      <c r="A477" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B477" t="inlineStr">
+        <is>
+          <t>Herbicida</t>
+        </is>
+      </c>
+      <c r="C477" t="inlineStr">
+        <is>
+          <t>GLIFOSATO</t>
+        </is>
+      </c>
+      <c r="D477" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="E477" t="n">
+        <v>33.67</v>
+      </c>
+      <c r="F477" t="inlineStr">
+        <is>
+          <t>Alface</t>
+        </is>
+      </c>
+      <c r="G477" t="n">
+        <v>2.28</v>
+      </c>
+    </row>
+    <row r="478">
+      <c r="A478" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B478" t="inlineStr">
+        <is>
+          <t>Herbicida</t>
+        </is>
+      </c>
+      <c r="C478" t="inlineStr">
+        <is>
+          <t>DIURON, 500 SC</t>
+        </is>
+      </c>
+      <c r="D478" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="E478" t="n">
+        <v>55.1</v>
+      </c>
+      <c r="F478" t="inlineStr">
+        <is>
+          <t>Banana</t>
+        </is>
+      </c>
+      <c r="G478" t="n">
+        <v>2.816</v>
+      </c>
+    </row>
+    <row r="479">
+      <c r="A479" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B479" t="inlineStr">
+        <is>
+          <t>Herbicida</t>
+        </is>
+      </c>
+      <c r="C479" t="inlineStr">
+        <is>
+          <t>2,4-D</t>
+        </is>
+      </c>
+      <c r="D479" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="E479" t="n">
+        <v>20.02</v>
+      </c>
+      <c r="F479" t="inlineStr">
+        <is>
+          <t>Banana</t>
+        </is>
+      </c>
+      <c r="G479" t="n">
+        <v>2.816</v>
+      </c>
+    </row>
+    <row r="480">
+      <c r="A480" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B480" t="inlineStr">
+        <is>
+          <t>Inseticida</t>
+        </is>
+      </c>
+      <c r="C480" t="inlineStr">
+        <is>
+          <t>ENGEO PLENO, 106 G/L, TIAMETOXAM, NEONICOTINÓIDE + PIRETRÓIDE, SC</t>
+        </is>
+      </c>
+      <c r="D480" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="E480" t="n">
+        <v>183.335</v>
+      </c>
+      <c r="F480" t="inlineStr">
+        <is>
+          <t>Banana</t>
+        </is>
+      </c>
+      <c r="G480" t="n">
+        <v>2.815833333333333</v>
+      </c>
+    </row>
+    <row r="481">
+      <c r="A481" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B481" t="inlineStr">
+        <is>
+          <t>Inseticida</t>
+        </is>
+      </c>
+      <c r="C481" t="inlineStr">
+        <is>
+          <t>CLORPIRIFÓS</t>
+        </is>
+      </c>
+      <c r="D481" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="E481" t="n">
+        <v>52.23999999999999</v>
+      </c>
+      <c r="F481" t="inlineStr">
+        <is>
+          <t>Alface</t>
+        </is>
+      </c>
+      <c r="G481" t="n">
+        <v>2.2805</v>
+      </c>
+    </row>
+    <row r="482">
+      <c r="A482" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B482" t="inlineStr">
+        <is>
+          <t>Inseticida</t>
+        </is>
+      </c>
+      <c r="C482" t="inlineStr">
+        <is>
+          <t>ENGEO PLENO, 106 G/L, TIAMETOXAM, NEONICOTINÓIDE + PIRETRÓIDE, SC</t>
+        </is>
+      </c>
+      <c r="D482" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="E482" t="n">
+        <v>183.335</v>
+      </c>
+      <c r="F482" t="inlineStr">
+        <is>
+          <t>Banana</t>
+        </is>
+      </c>
+      <c r="G482" t="n">
+        <v>2.815833333333333</v>
+      </c>
+    </row>
+    <row r="483">
+      <c r="A483" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B483" t="inlineStr">
+        <is>
+          <t>Inseticida</t>
+        </is>
+      </c>
+      <c r="C483" t="inlineStr">
+        <is>
+          <t>CLORPIRIFÓS</t>
+        </is>
+      </c>
+      <c r="D483" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="E483" t="n">
+        <v>52.23999999999999</v>
+      </c>
+      <c r="F483" t="inlineStr">
+        <is>
+          <t>Alface</t>
+        </is>
+      </c>
+      <c r="G483" t="n">
+        <v>2.2805</v>
+      </c>
+    </row>
+    <row r="484">
+      <c r="A484" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B484" t="inlineStr">
+        <is>
+          <t>Inseticida</t>
+        </is>
+      </c>
+      <c r="C484" t="inlineStr">
+        <is>
+          <t>CLORPIRIFÓS</t>
+        </is>
+      </c>
+      <c r="D484" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="E484" t="n">
+        <v>52.23999999999999</v>
+      </c>
+      <c r="F484" t="inlineStr">
+        <is>
+          <t>Alface</t>
+        </is>
+      </c>
+      <c r="G484" t="n">
+        <v>2.2805</v>
+      </c>
+    </row>
+    <row r="485">
+      <c r="A485" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B485" t="inlineStr">
+        <is>
+          <t>Inseticida</t>
+        </is>
+      </c>
+      <c r="C485" t="inlineStr">
+        <is>
+          <t>ENGEO PLENO, 106 G/L, TIAMETOXAM, NEONICOTINÓIDE + PIRETRÓIDE, SC</t>
+        </is>
+      </c>
+      <c r="D485" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="E485" t="n">
+        <v>183.335</v>
+      </c>
+      <c r="F485" t="inlineStr">
+        <is>
+          <t>Banana</t>
+        </is>
+      </c>
+      <c r="G485" t="n">
+        <v>2.815833333333333</v>
+      </c>
+    </row>
+    <row r="486">
+      <c r="A486" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B486" t="inlineStr">
+        <is>
+          <t>Inseticida</t>
+        </is>
+      </c>
+      <c r="C486" t="inlineStr">
+        <is>
+          <t>ENGEO PLENO, 106 G/L, TIAMETOXAM, NEONICOTINÓIDE + PIRETRÓIDE, SC</t>
+        </is>
+      </c>
+      <c r="D486" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="E486" t="n">
+        <v>183.335</v>
+      </c>
+      <c r="F486" t="inlineStr">
+        <is>
+          <t>Banana</t>
+        </is>
+      </c>
+      <c r="G486" t="n">
+        <v>2.815833333333333</v>
+      </c>
+    </row>
+    <row r="487">
+      <c r="A487" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B487" t="inlineStr">
+        <is>
+          <t>Inseticida</t>
+        </is>
+      </c>
+      <c r="C487" t="inlineStr">
+        <is>
+          <t>CLORPIRIFÓS</t>
+        </is>
+      </c>
+      <c r="D487" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="E487" t="n">
+        <v>52.23999999999999</v>
+      </c>
+      <c r="F487" t="inlineStr">
+        <is>
+          <t>Alface</t>
+        </is>
+      </c>
+      <c r="G487" t="n">
+        <v>2.2805</v>
+      </c>
+    </row>
+    <row r="488">
+      <c r="A488" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B488" t="inlineStr">
+        <is>
+          <t>Inseticida</t>
+        </is>
+      </c>
+      <c r="C488" t="inlineStr">
+        <is>
+          <t>ENGEO PLENO, 106 G/L, TIAMETOXAM, NEONICOTINÓIDE + PIRETRÓIDE, SC</t>
+        </is>
+      </c>
+      <c r="D488" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="E488" t="n">
+        <v>183.335</v>
+      </c>
+      <c r="F488" t="inlineStr">
+        <is>
+          <t>Banana</t>
+        </is>
+      </c>
+      <c r="G488" t="n">
+        <v>2.815833333333333</v>
+      </c>
+    </row>
+    <row r="489">
+      <c r="A489" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B489" t="inlineStr">
+        <is>
+          <t>Inseticida</t>
+        </is>
+      </c>
+      <c r="C489" t="inlineStr">
+        <is>
+          <t>CLORPIRIFÓS</t>
+        </is>
+      </c>
+      <c r="D489" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="E489" t="n">
+        <v>52.23999999999999</v>
+      </c>
+      <c r="F489" t="inlineStr">
+        <is>
+          <t>Alface</t>
+        </is>
+      </c>
+      <c r="G489" t="n">
+        <v>2.2805</v>
+      </c>
+    </row>
+    <row r="490">
+      <c r="A490" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B490" t="inlineStr">
+        <is>
+          <t>Inseticida</t>
+        </is>
+      </c>
+      <c r="C490" t="inlineStr">
+        <is>
+          <t>CLORPIRIFÓS</t>
+        </is>
+      </c>
+      <c r="D490" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="E490" t="n">
+        <v>52.23999999999999</v>
+      </c>
+      <c r="F490" t="inlineStr">
+        <is>
+          <t>Alface</t>
+        </is>
+      </c>
+      <c r="G490" t="n">
+        <v>2.2805</v>
+      </c>
+    </row>
+    <row r="491">
+      <c r="A491" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B491" t="inlineStr">
+        <is>
+          <t>Inseticida</t>
+        </is>
+      </c>
+      <c r="C491" t="inlineStr">
+        <is>
+          <t>ENGEO PLENO, 106 G/L, TIAMETOXAM, NEONICOTINÓIDE + PIRETRÓIDE, SC</t>
+        </is>
+      </c>
+      <c r="D491" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="E491" t="n">
+        <v>183.335</v>
+      </c>
+      <c r="F491" t="inlineStr">
+        <is>
+          <t>Banana</t>
+        </is>
+      </c>
+      <c r="G491" t="n">
+        <v>2.815833333333333</v>
+      </c>
+    </row>
+    <row r="492">
+      <c r="A492" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B492" t="inlineStr">
+        <is>
+          <t>Inseticida</t>
+        </is>
+      </c>
+      <c r="C492" t="inlineStr">
+        <is>
+          <t>ENGEO PLENO, 106 G/L, TIAMETOXAM, NEONICOTINÓIDE + PIRETRÓIDE, SC</t>
+        </is>
+      </c>
+      <c r="D492" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="E492" t="n">
+        <v>183.335</v>
+      </c>
+      <c r="F492" t="inlineStr">
+        <is>
+          <t>Banana</t>
+        </is>
+      </c>
+      <c r="G492" t="n">
+        <v>2.815833333333333</v>
+      </c>
+    </row>
+    <row r="493">
+      <c r="A493" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B493" t="inlineStr">
+        <is>
+          <t>Inseticida</t>
+        </is>
+      </c>
+      <c r="C493" t="inlineStr">
+        <is>
+          <t>CLORPIRIFÓS</t>
+        </is>
+      </c>
+      <c r="D493" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="E493" t="n">
+        <v>52.23999999999999</v>
+      </c>
+      <c r="F493" t="inlineStr">
+        <is>
+          <t>Alface</t>
+        </is>
+      </c>
+      <c r="G493" t="n">
+        <v>2.2805</v>
+      </c>
+    </row>
+    <row r="494">
+      <c r="A494" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B494" t="inlineStr">
+        <is>
+          <t>Inseticida</t>
+        </is>
+      </c>
+      <c r="C494" t="inlineStr">
+        <is>
+          <t>ENGEO PLENO, 106 G/L, TIAMETOXAM, NEONICOTINÓIDE + PIRETRÓIDE, SC</t>
+        </is>
+      </c>
+      <c r="D494" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="E494" t="n">
+        <v>183.335</v>
+      </c>
+      <c r="F494" t="inlineStr">
+        <is>
+          <t>Banana</t>
+        </is>
+      </c>
+      <c r="G494" t="n">
+        <v>2.815833333333333</v>
+      </c>
+    </row>
+    <row r="495">
+      <c r="A495" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B495" t="inlineStr">
+        <is>
+          <t>Inseticida</t>
+        </is>
+      </c>
+      <c r="C495" t="inlineStr">
+        <is>
+          <t>CLORPIRIFÓS</t>
+        </is>
+      </c>
+      <c r="D495" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="E495" t="n">
+        <v>52.23999999999999</v>
+      </c>
+      <c r="F495" t="inlineStr">
+        <is>
+          <t>Alface</t>
+        </is>
+      </c>
+      <c r="G495" t="n">
+        <v>2.2805</v>
+      </c>
+    </row>
+    <row r="496">
+      <c r="A496" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B496" t="inlineStr">
+        <is>
+          <t>Inseticida</t>
+        </is>
+      </c>
+      <c r="C496" t="inlineStr">
+        <is>
+          <t>CLORPIRIFÓS</t>
+        </is>
+      </c>
+      <c r="D496" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="E496" t="n">
+        <v>52.23999999999999</v>
+      </c>
+      <c r="F496" t="inlineStr">
+        <is>
+          <t>Alface</t>
+        </is>
+      </c>
+      <c r="G496" t="n">
+        <v>2.2805</v>
+      </c>
+    </row>
+    <row r="497">
+      <c r="A497" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B497" t="inlineStr">
+        <is>
+          <t>Inseticida</t>
+        </is>
+      </c>
+      <c r="C497" t="inlineStr">
+        <is>
+          <t>ENGEO PLENO, 106 G/L, TIAMETOXAM, NEONICOTINÓIDE + PIRETRÓIDE, SC</t>
+        </is>
+      </c>
+      <c r="D497" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="E497" t="n">
+        <v>183.335</v>
+      </c>
+      <c r="F497" t="inlineStr">
+        <is>
+          <t>Banana</t>
+        </is>
+      </c>
+      <c r="G497" t="n">
+        <v>2.815833333333333</v>
+      </c>
+    </row>
+    <row r="498">
+      <c r="A498" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B498" t="inlineStr">
+        <is>
+          <t>Inseticida</t>
+        </is>
+      </c>
+      <c r="C498" t="inlineStr">
+        <is>
+          <t>CLORPIRIFÓS</t>
+        </is>
+      </c>
+      <c r="D498" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="E498" t="n">
+        <v>52.23999999999999</v>
+      </c>
+      <c r="F498" t="inlineStr">
+        <is>
+          <t>Alface</t>
+        </is>
+      </c>
+      <c r="G498" t="n">
+        <v>2.2805</v>
+      </c>
+    </row>
+    <row r="499">
+      <c r="A499" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B499" t="inlineStr">
+        <is>
+          <t>Inseticida</t>
+        </is>
+      </c>
+      <c r="C499" t="inlineStr">
+        <is>
+          <t>ENGEO PLENO, 106 G/L, TIAMETOXAM, NEONICOTINÓIDE + PIRETRÓIDE, SC</t>
+        </is>
+      </c>
+      <c r="D499" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="E499" t="n">
+        <v>183.335</v>
+      </c>
+      <c r="F499" t="inlineStr">
+        <is>
+          <t>Banana</t>
+        </is>
+      </c>
+      <c r="G499" t="n">
+        <v>2.815833333333333</v>
+      </c>
+    </row>
+    <row r="500">
+      <c r="A500" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B500" t="inlineStr">
+        <is>
+          <t>Inseticida</t>
+        </is>
+      </c>
+      <c r="C500" t="inlineStr">
+        <is>
+          <t>CLORPIRIFÓS</t>
+        </is>
+      </c>
+      <c r="D500" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="E500" t="n">
+        <v>52.23999999999999</v>
+      </c>
+      <c r="F500" t="inlineStr">
+        <is>
+          <t>Alface</t>
+        </is>
+      </c>
+      <c r="G500" t="n">
+        <v>2.2805</v>
+      </c>
+    </row>
+    <row r="501">
+      <c r="A501" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B501" t="inlineStr">
+        <is>
+          <t>Inseticida</t>
+        </is>
+      </c>
+      <c r="C501" t="inlineStr">
+        <is>
+          <t>ENGEO PLENO, 106 G/L, TIAMETOXAM, NEONICOTINÓIDE + PIRETRÓIDE, SC</t>
+        </is>
+      </c>
+      <c r="D501" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="E501" t="n">
+        <v>183.335</v>
+      </c>
+      <c r="F501" t="inlineStr">
+        <is>
+          <t>Banana</t>
+        </is>
+      </c>
+      <c r="G501" t="n">
+        <v>2.815833333333333</v>
+      </c>
+    </row>
+    <row r="502">
+      <c r="A502" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B502" t="inlineStr">
+        <is>
+          <t>Inseticida</t>
+        </is>
+      </c>
+      <c r="C502" t="inlineStr">
+        <is>
+          <t>ENGEO PLENO, 106 G/L, TIAMETOXAM, NEONICOTINÓIDE + PIRETRÓIDE, SC</t>
+        </is>
+      </c>
+      <c r="D502" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="E502" t="n">
+        <v>183.335</v>
+      </c>
+      <c r="F502" t="inlineStr">
+        <is>
+          <t>Banana</t>
+        </is>
+      </c>
+      <c r="G502" t="n">
+        <v>2.8175</v>
+      </c>
+    </row>
+    <row r="503">
+      <c r="A503" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B503" t="inlineStr">
+        <is>
+          <t>Inseticida</t>
+        </is>
+      </c>
+      <c r="C503" t="inlineStr">
+        <is>
+          <t>IMIDACLOPRID 700, 700 G/KG, IMIDACLOPRIDO, NEONICOTINÓIDE, WG</t>
+        </is>
+      </c>
+      <c r="D503" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="E503" t="n">
+        <v>113.81</v>
+      </c>
+      <c r="F503" t="inlineStr">
+        <is>
+          <t>Alface</t>
+        </is>
+      </c>
+      <c r="G503" t="n">
+        <v>2.288694444444444</v>
+      </c>
+    </row>
+    <row r="504">
+      <c r="A504" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B504" t="inlineStr">
+        <is>
+          <t>Inseticida</t>
+        </is>
+      </c>
+      <c r="C504" t="inlineStr">
+        <is>
+          <t>CLORPIRIFÓS</t>
+        </is>
+      </c>
+      <c r="D504" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="E504" t="n">
+        <v>52.23999999999999</v>
+      </c>
+      <c r="F504" t="inlineStr">
+        <is>
+          <t>Alface</t>
+        </is>
+      </c>
+      <c r="G504" t="n">
+        <v>2.288694444444444</v>
+      </c>
+    </row>
+    <row r="505">
+      <c r="A505" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B505" t="inlineStr">
+        <is>
+          <t>Herbicida</t>
+        </is>
+      </c>
+      <c r="C505" t="inlineStr">
+        <is>
+          <t>GLIFOSATO</t>
+        </is>
+      </c>
+      <c r="D505" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="E505" t="n">
+        <v>33.67</v>
+      </c>
+      <c r="F505" t="inlineStr">
+        <is>
+          <t>Alface</t>
+        </is>
+      </c>
+      <c r="G505" t="n">
+        <v>2.289</v>
+      </c>
+    </row>
+    <row r="506">
+      <c r="A506" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B506" t="inlineStr">
+        <is>
+          <t>Herbicida</t>
+        </is>
+      </c>
+      <c r="C506" t="inlineStr">
+        <is>
+          <t>DIURON, 500 SC</t>
+        </is>
+      </c>
+      <c r="D506" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="E506" t="n">
+        <v>55.1</v>
+      </c>
+      <c r="F506" t="inlineStr">
+        <is>
+          <t>Banana</t>
+        </is>
+      </c>
+      <c r="G506" t="n">
+        <v>2.817</v>
+      </c>
+    </row>
+    <row r="507">
+      <c r="A507" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B507" t="inlineStr">
+        <is>
+          <t>Herbicida</t>
+        </is>
+      </c>
+      <c r="C507" t="inlineStr">
+        <is>
+          <t>2,4-D</t>
+        </is>
+      </c>
+      <c r="D507" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="E507" t="n">
+        <v>20.02</v>
+      </c>
+      <c r="F507" t="inlineStr">
+        <is>
+          <t>Banana</t>
+        </is>
+      </c>
+      <c r="G507" t="n">
+        <v>2.817</v>
+      </c>
+    </row>
+    <row r="508">
+      <c r="A508" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B508" t="inlineStr">
+        <is>
+          <t>Inseticida</t>
+        </is>
+      </c>
+      <c r="C508" t="inlineStr">
+        <is>
+          <t>ENGEO PLENO, 106 G/L, TIAMETOXAM, NEONICOTINÓIDE + PIRETRÓIDE, SC</t>
+        </is>
+      </c>
+      <c r="D508" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="E508" t="n">
+        <v>183.335</v>
+      </c>
+      <c r="F508" t="inlineStr">
+        <is>
+          <t>Banana</t>
+        </is>
+      </c>
+      <c r="G508" t="n">
+        <v>2.8175</v>
+      </c>
+    </row>
+    <row r="509">
+      <c r="A509" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B509" t="inlineStr">
+        <is>
+          <t>Inseticida</t>
+        </is>
+      </c>
+      <c r="C509" t="inlineStr">
+        <is>
+          <t>CLORPIRIFÓS</t>
+        </is>
+      </c>
+      <c r="D509" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="E509" t="n">
+        <v>52.23999999999999</v>
+      </c>
+      <c r="F509" t="inlineStr">
+        <is>
+          <t>Alface</t>
+        </is>
+      </c>
+      <c r="G509" t="n">
+        <v>2.288694444444444</v>
+      </c>
+    </row>
+    <row r="510">
+      <c r="A510" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B510" t="inlineStr">
+        <is>
+          <t>Inseticida</t>
+        </is>
+      </c>
+      <c r="C510" t="inlineStr">
+        <is>
+          <t>IMIDACLOPRID 700, 700 G/KG, IMIDACLOPRIDO, NEONICOTINÓIDE, WG</t>
+        </is>
+      </c>
+      <c r="D510" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="E510" t="n">
+        <v>113.81</v>
+      </c>
+      <c r="F510" t="inlineStr">
+        <is>
+          <t>Alface</t>
+        </is>
+      </c>
+      <c r="G510" t="n">
+        <v>2.288694444444444</v>
+      </c>
+    </row>
+    <row r="511">
+      <c r="A511" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B511" t="inlineStr">
+        <is>
+          <t>Inseticida</t>
+        </is>
+      </c>
+      <c r="C511" t="inlineStr">
+        <is>
+          <t>ENGEO PLENO, 106 G/L, TIAMETOXAM, NEONICOTINÓIDE + PIRETRÓIDE, SC</t>
+        </is>
+      </c>
+      <c r="D511" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="E511" t="n">
+        <v>183.335</v>
+      </c>
+      <c r="F511" t="inlineStr">
+        <is>
+          <t>Banana</t>
+        </is>
+      </c>
+      <c r="G511" t="n">
+        <v>2.8175</v>
+      </c>
+    </row>
+    <row r="512">
+      <c r="A512" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B512" t="inlineStr">
+        <is>
+          <t>Inseticida</t>
+        </is>
+      </c>
+      <c r="C512" t="inlineStr">
+        <is>
+          <t>CLORPIRIFÓS</t>
+        </is>
+      </c>
+      <c r="D512" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="E512" t="n">
+        <v>52.23999999999999</v>
+      </c>
+      <c r="F512" t="inlineStr">
+        <is>
+          <t>Alface</t>
+        </is>
+      </c>
+      <c r="G512" t="n">
+        <v>2.288694444444444</v>
+      </c>
+    </row>
+    <row r="513">
+      <c r="A513" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B513" t="inlineStr">
+        <is>
+          <t>Inseticida</t>
+        </is>
+      </c>
+      <c r="C513" t="inlineStr">
+        <is>
+          <t>IMIDACLOPRID 700, 700 G/KG, IMIDACLOPRIDO, NEONICOTINÓIDE, WG</t>
+        </is>
+      </c>
+      <c r="D513" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="E513" t="n">
+        <v>113.81</v>
+      </c>
+      <c r="F513" t="inlineStr">
+        <is>
+          <t>Alface</t>
+        </is>
+      </c>
+      <c r="G513" t="n">
+        <v>2.288694444444444</v>
+      </c>
+    </row>
+    <row r="514">
+      <c r="A514" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B514" t="inlineStr">
+        <is>
+          <t>Inseticida</t>
+        </is>
+      </c>
+      <c r="C514" t="inlineStr">
+        <is>
+          <t>IMIDACLOPRID 700, 700 G/KG, IMIDACLOPRIDO, NEONICOTINÓIDE, WG</t>
+        </is>
+      </c>
+      <c r="D514" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="E514" t="n">
+        <v>113.81</v>
+      </c>
+      <c r="F514" t="inlineStr">
+        <is>
+          <t>Alface</t>
+        </is>
+      </c>
+      <c r="G514" t="n">
+        <v>2.288694444444444</v>
+      </c>
+    </row>
+    <row r="515">
+      <c r="A515" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B515" t="inlineStr">
+        <is>
+          <t>Inseticida</t>
+        </is>
+      </c>
+      <c r="C515" t="inlineStr">
+        <is>
+          <t>CLORPIRIFÓS</t>
+        </is>
+      </c>
+      <c r="D515" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="E515" t="n">
+        <v>52.23999999999999</v>
+      </c>
+      <c r="F515" t="inlineStr">
+        <is>
+          <t>Alface</t>
+        </is>
+      </c>
+      <c r="G515" t="n">
+        <v>2.288694444444444</v>
+      </c>
+    </row>
+    <row r="516">
+      <c r="A516" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B516" t="inlineStr">
+        <is>
+          <t>Inseticida</t>
+        </is>
+      </c>
+      <c r="C516" t="inlineStr">
+        <is>
+          <t>ENGEO PLENO, 106 G/L, TIAMETOXAM, NEONICOTINÓIDE + PIRETRÓIDE, SC</t>
+        </is>
+      </c>
+      <c r="D516" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="E516" t="n">
+        <v>183.335</v>
+      </c>
+      <c r="F516" t="inlineStr">
+        <is>
+          <t>Banana</t>
+        </is>
+      </c>
+      <c r="G516" t="n">
+        <v>2.8175</v>
+      </c>
+    </row>
+    <row r="517">
+      <c r="A517" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B517" t="inlineStr">
+        <is>
+          <t>Inseticida</t>
+        </is>
+      </c>
+      <c r="C517" t="inlineStr">
+        <is>
+          <t>IMIDACLOPRID 700, 700 G/KG, IMIDACLOPRIDO, NEONICOTINÓIDE, WG</t>
+        </is>
+      </c>
+      <c r="D517" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="E517" t="n">
+        <v>113.81</v>
+      </c>
+      <c r="F517" t="inlineStr">
+        <is>
+          <t>Alface</t>
+        </is>
+      </c>
+      <c r="G517" t="n">
+        <v>2.288694444444444</v>
+      </c>
+    </row>
+    <row r="518">
+      <c r="A518" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B518" t="inlineStr">
+        <is>
+          <t>Inseticida</t>
+        </is>
+      </c>
+      <c r="C518" t="inlineStr">
+        <is>
+          <t>CLORPIRIFÓS</t>
+        </is>
+      </c>
+      <c r="D518" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="E518" t="n">
+        <v>52.23999999999999</v>
+      </c>
+      <c r="F518" t="inlineStr">
+        <is>
+          <t>Alface</t>
+        </is>
+      </c>
+      <c r="G518" t="n">
+        <v>2.288694444444444</v>
+      </c>
+    </row>
+    <row r="519">
+      <c r="A519" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B519" t="inlineStr">
+        <is>
+          <t>Inseticida</t>
+        </is>
+      </c>
+      <c r="C519" t="inlineStr">
+        <is>
+          <t>ENGEO PLENO, 106 G/L, TIAMETOXAM, NEONICOTINÓIDE + PIRETRÓIDE, SC</t>
+        </is>
+      </c>
+      <c r="D519" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="E519" t="n">
+        <v>183.335</v>
+      </c>
+      <c r="F519" t="inlineStr">
+        <is>
+          <t>Banana</t>
+        </is>
+      </c>
+      <c r="G519" t="n">
+        <v>2.8175</v>
+      </c>
+    </row>
+    <row r="520">
+      <c r="A520" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B520" t="inlineStr">
+        <is>
+          <t>Inseticida</t>
+        </is>
+      </c>
+      <c r="C520" t="inlineStr">
+        <is>
+          <t>ENGEO PLENO, 106 G/L, TIAMETOXAM, NEONICOTINÓIDE + PIRETRÓIDE, SC</t>
+        </is>
+      </c>
+      <c r="D520" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="E520" t="n">
+        <v>183.335</v>
+      </c>
+      <c r="F520" t="inlineStr">
+        <is>
+          <t>Banana</t>
+        </is>
+      </c>
+      <c r="G520" t="n">
+        <v>2.949583333333333</v>
+      </c>
+    </row>
+    <row r="521">
+      <c r="A521" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B521" t="inlineStr">
+        <is>
+          <t>Inseticida</t>
+        </is>
+      </c>
+      <c r="C521" t="inlineStr">
+        <is>
+          <t>IMIDACLOPRID 700, 700 G/KG, IMIDACLOPRIDO, NEONICOTINÓIDE, WG</t>
+        </is>
+      </c>
+      <c r="D521" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="E521" t="n">
+        <v>113.81</v>
+      </c>
+      <c r="F521" t="inlineStr">
+        <is>
+          <t>Alface</t>
+        </is>
+      </c>
+      <c r="G521" t="n">
+        <v>2.346611111111111</v>
+      </c>
+    </row>
+    <row r="522">
+      <c r="A522" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B522" t="inlineStr">
+        <is>
+          <t>Inseticida</t>
+        </is>
+      </c>
+      <c r="C522" t="inlineStr">
+        <is>
+          <t>CLORPIRIFÓS</t>
+        </is>
+      </c>
+      <c r="D522" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="E522" t="n">
+        <v>52.23999999999999</v>
+      </c>
+      <c r="F522" t="inlineStr">
+        <is>
+          <t>Alface</t>
+        </is>
+      </c>
+      <c r="G522" t="n">
+        <v>2.346611111111111</v>
+      </c>
+    </row>
+    <row r="523">
+      <c r="A523" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B523" t="inlineStr">
+        <is>
+          <t>Herbicida</t>
+        </is>
+      </c>
+      <c r="C523" t="inlineStr">
+        <is>
+          <t>2,4-D</t>
+        </is>
+      </c>
+      <c r="D523" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="E523" t="n">
+        <v>20.02</v>
+      </c>
+      <c r="F523" t="inlineStr">
+        <is>
+          <t>Banana</t>
+        </is>
+      </c>
+      <c r="G523" t="n">
+        <v>2.95</v>
+      </c>
+    </row>
+    <row r="524">
+      <c r="A524" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B524" t="inlineStr">
+        <is>
+          <t>Herbicida</t>
+        </is>
+      </c>
+      <c r="C524" t="inlineStr">
+        <is>
+          <t>GLIFOSATO</t>
+        </is>
+      </c>
+      <c r="D524" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="E524" t="n">
+        <v>33.67</v>
+      </c>
+      <c r="F524" t="inlineStr">
+        <is>
+          <t>Alface</t>
+        </is>
+      </c>
+      <c r="G524" t="n">
+        <v>2.347</v>
+      </c>
+    </row>
+    <row r="525">
+      <c r="A525" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B525" t="inlineStr">
+        <is>
+          <t>Herbicida</t>
+        </is>
+      </c>
+      <c r="C525" t="inlineStr">
+        <is>
+          <t>DIURON, 500 SC</t>
+        </is>
+      </c>
+      <c r="D525" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="E525" t="n">
+        <v>55.1</v>
+      </c>
+      <c r="F525" t="inlineStr">
+        <is>
+          <t>Banana</t>
+        </is>
+      </c>
+      <c r="G525" t="n">
+        <v>2.95</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>